<commit_message>
chore: bump version to v21.5.5 in codebase and repository checklist
</commit_message>
<xml_diff>
--- a/checklist_homologacao.xlsx
+++ b/checklist_homologacao.xlsx
@@ -880,7 +880,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Aprovado na v2.6.2: Alterado de 'Até 2 pessoas cuidadas' para 'Até 1 pessoa cuidada' no card de preços e no javascript do site.</t>
+          <t>Aprovado na v21.5.5: Alterado de 'Até 2 pessoas cuidadas' para 'Até 1 pessoa cuidada' no card de preços e no javascript do site.</t>
         </is>
       </c>
       <c r="G13" s="3" t="n"/>
@@ -915,7 +915,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Aprovado na v2.6.2: O botão 'Testar grátis' foi estilizado com a cor amarela/ouro (.btn-warning) para alta visibilidade e alinhamento visual.</t>
+          <t>Aprovado na v21.5.5: O botão 'Testar grátis' foi estilizado com a cor amarela/ouro (.btn-warning) para alta visibilidade e alinhamento visual.</t>
         </is>
       </c>
       <c r="G14" s="5" t="n"/>
@@ -950,7 +950,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Aprovado na v2.6.2: O recurso 'Falar com a Equipe' está totalmente implementado via chat com IA e integrado à API do backend.</t>
+          <t>Aprovado na v21.5.5: O recurso 'Falar com a Equipe' está totalmente implementado via chat com IA e integrado à API do backend.</t>
         </is>
       </c>
       <c r="G15" s="3" t="n"/>
@@ -985,7 +985,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Aprovado na v2.6.2: Ficha Médica agora possui slots e visualização separados para Frente e Verso dos documentos (RG/CPF e Carteirinha).</t>
+          <t>Aprovado na v21.5.5: Ficha Médica agora possui slots e visualização separados para Frente e Verso dos documentos (RG/CPF e Carteirinha).</t>
         </is>
       </c>
       <c r="G16" s="5" t="n"/>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Aprovado na v2.6.2: Tratamento robusto para MIME types genéricos (como octet-stream no celular) adicionado aos endpoints de upload e OCR.</t>
+          <t>Aprovado na v21.5.5: Tratamento robusto para MIME types genéricos (como octet-stream no celular) adicionado aos endpoints de upload e OCR.</t>
         </is>
       </c>
       <c r="G17" s="3" t="n"/>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Aprovado na v2.6.2: O envio de documentos por e-mail foi atualizado para ler os múltiplos arquivos e anexar Frente e Verso separadamente.</t>
+          <t>Aprovado na v21.5.5: O envio de documentos por e-mail foi atualizado para ler os múltiplos arquivos e anexar Frente e Verso separadamente.</t>
         </is>
       </c>
       <c r="G18" s="5" t="n"/>

</xml_diff>

<commit_message>
doc: add new test cases CT-021 to CT-027 to checklist for document uploads, support chatbot on landing page, and clock picker customization
</commit_message>
<xml_diff>
--- a/checklist_homologacao.xlsx
+++ b/checklist_homologacao.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="7" min="1" max="1"/>
@@ -1180,6 +1180,277 @@
       <c r="F22" s="4" t="n"/>
       <c r="G22" s="5" t="n"/>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CT-021</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Ficha Médica (Cliente)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Anexar RG/CPF - Frente</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>1. Abrir a Ficha Médica (ícone de perfil 👤).
+2. No campo "Documento de Identidade (Frente)", selecionar e fazer o upload da foto da Frente.
+3. Clicar em "💾 Salvar".</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>O arquivo da Frente é enviado com sucesso e sua miniatura correspondente é exibida no preview da Ficha Médica.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Novo teste para homologação dos slots de anexos separados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CT-022</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Ficha Médica (Cliente)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Anexar RG/CPF - Verso</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>1. Abrir a Ficha Médica.
+2. No campo "Documento de Identidade (Verso)", selecionar e fazer o upload da foto do Verso.
+3. Clicar em "💾 Salvar".</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>O arquivo do Verso é armazenado separadamente da Frente e sua miniatura aparece de forma independente no preview.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Novo teste para homologação dos slots de anexos separados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CT-023</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Ficha Médica (Cliente)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Anexar Carteirinha de Saúde - Frente (com OCR)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>1. Abrir a Ficha Médica.
+2. No campo "Carteirinha de Convênio (Frente)", fazer o upload do documento.
+3. Aguardar a leitura por OCR e clicar em "💾 Salvar".</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>A imagem da Frente é salva, a miniatura é exibida, e o OCR do Gemini lê a operadora e matrícula preenchendo automaticamente o campo de texto.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Novo teste para homologação dos slots de anexos separados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CT-024</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Ficha Médica (Cliente)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Anexar Carteirinha de Saúde - Verso</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>1. Abrir a Ficha Médica.
+2. No campo "Carteirinha de Convênio (Verso)", fazer o upload do documento e clicar em "💾 Salvar".</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>O arquivo do Verso é armazenado com sucesso no backend de forma independente e sua miniatura correspondente é exibida no preview.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Novo teste para homologação dos slots de anexos separados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CT-025</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Landing Page (index.html)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Botão Falar com a Equipe (Chat IA)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>1. Acessar a página inicial do site.
+2. Clicar no botão "Falar com a equipe" do banner principal.
+3. Enviar uma mensagem comum (ex: "Qual é o preço do plano Pro?").</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>A modal de suporte abre imediatamente em vez de voltar ao início da página e o Maximus responde usando a IA do Gemini.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Novo teste para homologação da integração do chat IA na landing page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CT-026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Landing Page (index.html)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Falar com a Equipe - Escalação de Protocolo</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>1. Na modal de suporte, enviar uma dúvida complexa ou fora de escopo (ex: "Quero agendar uma visita presencial para reclamação").
+2. Verificar a geração de protocolo.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>O sistema responde com a mensagem de que a dúvida foi escalada, gera o número de protocolo em tela e encaminha o e-mail de suporte.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Novo teste para homologação do fluxo de escalação por e-mail de visitantes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CT-027</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Ficha Médica (Cliente)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Horário de Relatório Diário (Seletor Personalizado)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>1. Abrir a Ficha Médica para edição.
+2. No campo "Horário de Envio para o Responsável", usar os seletores de Horas (00-23) e Minutos (00-59).
+3. Salvar e conferir após recarregar.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Os seletores dropdowns aparecem listados para seleção simples (sem o widget de relógio radial do navegador) e salvam o horário com sucesso.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Novo teste para homologação da substituição do relógio de círculos radiais por select dropdowns.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>